<commit_message>
chore(tracker): record what the filter glyph took to get right
Updated the existing header row's note rather than adding a near-duplicate row.
The lesson is the transferable part: a glyph must be judged at the size and
density it ships at. A 390px screenshot showed only that a button existed, which
is how a hamburger survived a pass I reported as verified.

Unassigned still 0, OVERALL 242/267.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SportIQ-Delivery-Board.xlsx
+++ b/SportIQ-Delivery-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\IdeaProjects\SportIQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5495D80D-38CB-4ABD-BDBA-E8AB08AD87A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0114D2E5-1899-413B-8F2E-5B47F6726F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2371,7 +2371,7 @@
     <t>Picks header: wordmark left, one filter control carrying an off-default dot</t>
   </si>
   <si>
-    <t>The dot is the point -- a card can vanish because a slider sits where the user left it days ago, and with controls behind a sheet nothing said so. Theme toggle and hub button removed only after confirming both are still reachable from Profile.</t>
+    <t>The dot is the point -- a card can vanish because a slider sits where the user left it days ago, and with controls behind a sheet nothing said so. Theme toggle and hub button removed only after confirming both are still reachable from Profile. THE GLYPH TOOK TWO CORRECTIONS, both reported from a device: the spec's own "three stacked bars of descending width" was built and read as a hamburger, because stacked horizontal lines mean navigation whatever their widths; and three slider tracks left ~4px of air in a 36px button. Now two tracks with offset handles at 7 on 19 -- a handle over ~40% of its track reads as a toggle, not a slider. A glyph must be judged at the size and density it ships at; a 390px screenshot shows only that a button exists.</t>
   </si>
   <si>
     <t>Form chips re-coloured to clear AA contrast</t>
@@ -14329,7 +14329,7 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="258" spans="1:18" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="258" spans="1:18" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A258" t="s">
         <v>282</v>
       </c>
@@ -14359,7 +14359,7 @@
         <v>E6 Picks</v>
       </c>
     </row>
-    <row r="259" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="259" spans="1:18" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B259" t="s">
         <v>750</v>
       </c>
@@ -14386,7 +14386,7 @@
         <v>E6 Picks</v>
       </c>
     </row>
-    <row r="260" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="260" spans="1:18" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A260" t="s">
         <v>292</v>
       </c>
@@ -14416,7 +14416,7 @@
         <v>E7 Mobile</v>
       </c>
     </row>
-    <row r="261" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="261" spans="1:18" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B261" t="s">
         <v>755</v>
       </c>
@@ -14443,7 +14443,7 @@
         <v>E7 Mobile</v>
       </c>
     </row>
-    <row r="262" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="262" spans="1:18" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A262" t="s">
         <v>308</v>
       </c>
@@ -14473,7 +14473,7 @@
         <v>E8 Model Quality</v>
       </c>
     </row>
-    <row r="263" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="263" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A263" t="s">
         <v>369</v>
       </c>
@@ -14503,7 +14503,7 @@
         <v>E10 Deploy</v>
       </c>
     </row>
-    <row r="264" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="264" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A264" t="s">
         <v>282</v>
       </c>
@@ -14533,7 +14533,7 @@
         <v>E6 Picks</v>
       </c>
     </row>
-    <row r="265" spans="1:18" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="265" spans="1:18" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A265" t="s">
         <v>398</v>
       </c>
@@ -14563,7 +14563,7 @@
         <v>E11 Ops Resilience</v>
       </c>
     </row>
-    <row r="266" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="266" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A266" t="s">
         <v>240</v>
       </c>
@@ -14593,7 +14593,7 @@
         <v>E2 Ingestion</v>
       </c>
     </row>
-    <row r="267" spans="1:18" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+    <row r="267" spans="1:18" ht="43.2" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A267" t="s">
         <v>338</v>
       </c>
@@ -14623,7 +14623,7 @@
         <v>E9 Data Ops</v>
       </c>
     </row>
-    <row r="268" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="268" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A268" t="s">
         <v>292</v>
       </c>
@@ -14653,7 +14653,7 @@
         <v>E7 Mobile</v>
       </c>
     </row>
-    <row r="269" spans="1:18" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+    <row r="269" spans="1:18" ht="57.6" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B269" t="s">
         <v>776</v>
       </c>
@@ -14680,7 +14680,7 @@
         <v>E7 Mobile</v>
       </c>
     </row>
-    <row r="270" spans="1:18" ht="72" x14ac:dyDescent="0.55000000000000004">
+    <row r="270" spans="1:18" ht="72" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B270" t="s">
         <v>778</v>
       </c>
@@ -14707,7 +14707,7 @@
         <v>E7 Mobile</v>
       </c>
     </row>
-    <row r="271" spans="1:18" ht="100.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="271" spans="1:18" ht="100.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A271" t="s">
         <v>369</v>
       </c>
@@ -15648,11 +15648,11 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="H14:M14"/>
     <mergeCell ref="N27:P27"/>
     <mergeCell ref="A26:S26"/>
+    <mergeCell ref="H20:M20"/>
     <mergeCell ref="A16:S16"/>
-    <mergeCell ref="H20:M20"/>
     <mergeCell ref="N20:S20"/>
     <mergeCell ref="A7:S7"/>
     <mergeCell ref="N11:P11"/>
@@ -15661,14 +15661,13 @@
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="K11:M11"/>
-    <mergeCell ref="B12:S12"/>
+    <mergeCell ref="B18:S18"/>
     <mergeCell ref="B6:S6"/>
     <mergeCell ref="Q11:S11"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B15:S15"/>
     <mergeCell ref="H5:J5"/>
-    <mergeCell ref="H14:M14"/>
     <mergeCell ref="A31:S31"/>
     <mergeCell ref="K39:M39"/>
     <mergeCell ref="A34:S34"/>
@@ -15677,6 +15676,7 @@
     <mergeCell ref="Q17:S17"/>
     <mergeCell ref="A30:S30"/>
     <mergeCell ref="A36:S36"/>
+    <mergeCell ref="H23:J23"/>
     <mergeCell ref="A37:S37"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="Q39:S39"/>
@@ -15684,7 +15684,7 @@
     <mergeCell ref="H39:J39"/>
     <mergeCell ref="N39:P39"/>
     <mergeCell ref="B8:J8"/>
-    <mergeCell ref="B18:S18"/>
+    <mergeCell ref="B12:S12"/>
     <mergeCell ref="A35:S35"/>
     <mergeCell ref="A4:S4"/>
     <mergeCell ref="H17:J17"/>
@@ -17676,7 +17676,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="95" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="95" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A95" s="214" t="s">
         <v>206</v>
       </c>
@@ -17693,7 +17693,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+    <row r="96" spans="1:5" ht="28.8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A96" s="214" t="s">
         <v>208</v>
       </c>

</xml_diff>